<commit_message>
add task 4 and others task
</commit_message>
<xml_diff>
--- a/PBQ – Organisasi Kecil Mengalami Phishing + Account Takeover____.xlsx
+++ b/PBQ – Organisasi Kecil Mengalami Phishing + Account Takeover____.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\Cyber Security\tugas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BC812F-6F48-4E5F-9F0E-4B0E169454F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="PBQ_Phishing_ATO" sheetId="1" r:id="rId5"/>
+    <sheet name="PBQ_Phishing_ATO" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="145">
   <si>
     <t>PBQ – Organisasi Kecil Mengalami Phishing + Account Takeover</t>
   </si>
@@ -365,9 +374,6 @@
     <t>Tidak ada phishing awareness training</t>
   </si>
   <si>
-    <t>karena</t>
-  </si>
-  <si>
     <t>Tidak ada attachment scanning</t>
   </si>
   <si>
@@ -421,18 +427,18 @@
   <si>
     <r>
       <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <i/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>Password policy</t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve"> lebih kuat</t>
     </r>
@@ -452,26 +458,26 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve">Simulasi </t>
     </r>
     <r>
       <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <i/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve">phishing </t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>berkala</t>
     </r>
@@ -485,26 +491,26 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve">Alert </t>
     </r>
     <r>
       <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <i/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve">login </t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>tidak biasa</t>
     </r>
@@ -522,48 +528,60 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="14.0"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
-    <font/>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="5">
@@ -571,7 +589,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -593,58 +611,92 @@
     </fill>
   </fills>
   <borders count="13">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF9E9E9E"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF9E9E9E"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF9E9E9E"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF9E9E9E"/>
       </right>
       <top style="thin">
         <color rgb="FF9E9E9E"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF9E9E9E"/>
       </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF9E9E9E"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF9E9E9E"/>
       </left>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FF9E9E9E"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FF9E9E9E"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF9E9E9E"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF9E9E9E"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -659,27 +711,34 @@
       <bottom style="thin">
         <color rgb="FF9E9E9E"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF9E9E9E"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF9E9E9E"/>
       </top>
       <bottom style="thin">
         <color rgb="FF9E9E9E"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF9E9E9E"/>
       </top>
       <bottom style="thin">
         <color rgb="FF9E9E9E"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF9E9E9E"/>
       </right>
@@ -689,80 +748,69 @@
       <bottom style="thin">
         <color rgb="FF9E9E9E"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="21">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="9" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="9" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="12" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="10" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -952,1396 +1000,1437 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M1071"/>
+  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="5.0"/>
-    <col customWidth="1" min="2" max="2" width="20.0"/>
-    <col customWidth="1" min="3" max="3" width="55.0"/>
-    <col customWidth="1" hidden="1" min="4" max="4" width="28.0"/>
-    <col customWidth="1" min="5" max="5" width="76.71"/>
-    <col customWidth="1" min="6" max="8" width="8.71"/>
-    <col customWidth="1" min="9" max="9" width="36.29"/>
-    <col customWidth="1" hidden="1" min="10" max="13" width="30.0"/>
-    <col customWidth="1" min="14" max="26" width="8.71"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="4" max="4" width="28" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="76.73046875" customWidth="1"/>
+    <col min="6" max="8" width="8.73046875" customWidth="1"/>
+    <col min="9" max="9" width="36.265625" customWidth="1"/>
+    <col min="10" max="13" width="30" hidden="1" customWidth="1"/>
+    <col min="14" max="26" width="8.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:13" ht="18">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="2" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+    </row>
+    <row r="2" spans="1:13" ht="14.25">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:13" ht="14.25">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4">
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:13" ht="14.25">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:13" ht="14.25">
+      <c r="A5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="7"/>
-      <c r="J5" s="3" t="s">
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8"/>
-      <c r="E6" s="9"/>
-      <c r="J6" s="3" t="s">
+    <row r="6" spans="1:13" ht="14.25">
+      <c r="A6" s="11"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8"/>
-      <c r="E7" s="9"/>
-      <c r="J7" s="3" t="s">
+    <row r="7" spans="1:13" ht="14.25">
+      <c r="A7" s="11"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L7" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8"/>
-      <c r="E8" s="9"/>
-      <c r="J8" s="3" t="s">
+    <row r="8" spans="1:13" ht="14.25">
+      <c r="A8" s="11"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="L8" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8"/>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" ht="54.75" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="12"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="s">
+    <row r="9" spans="1:13" ht="14.25">
+      <c r="A9" s="11"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+    </row>
+    <row r="10" spans="1:13" ht="54.75" customHeight="1">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:13" ht="14.25">
+      <c r="A11" s="17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" spans="1:13" ht="28.5">
+      <c r="A12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="16" t="s">
+    <row r="13" spans="1:13" ht="14.25">
+      <c r="A13" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="18"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="19">
-        <v>1.0</v>
-      </c>
-      <c r="B14" s="20" t="s">
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="20"/>
+    </row>
+    <row r="14" spans="1:13" ht="14.25">
+      <c r="A14" s="3">
+        <v>1</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="19"/>
-      <c r="E14" s="20"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="19">
-        <v>2.0</v>
-      </c>
-      <c r="B15" s="20" t="s">
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" spans="1:13" ht="14.25">
+      <c r="A15" s="3">
+        <v>2</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="19"/>
-      <c r="E15" s="20"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="19">
-        <v>3.0</v>
-      </c>
-      <c r="B16" s="20" t="s">
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" spans="1:13" ht="14.25">
+      <c r="A16" s="3">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="20"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="19">
-        <v>4.0</v>
-      </c>
-      <c r="B17" s="20" t="s">
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" ht="14.25">
+      <c r="A17" s="3">
+        <v>4</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="19"/>
-      <c r="E17" s="20"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="19">
-        <v>5.0</v>
-      </c>
-      <c r="B18" s="20" t="s">
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" ht="14.25">
+      <c r="A18" s="3">
+        <v>5</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="20"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="20">
-        <v>6.0</v>
-      </c>
-      <c r="B19" s="20" t="s">
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" ht="14.25">
+      <c r="A19" s="3">
+        <v>6</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="19"/>
-      <c r="E19" s="20"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="19">
-        <v>7.0</v>
-      </c>
-      <c r="B20" s="20" t="s">
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" ht="14.25">
+      <c r="A20" s="3">
+        <v>7</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="19"/>
-      <c r="E20" s="20"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="20">
-        <v>8.0</v>
-      </c>
-      <c r="B21" s="20" t="s">
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" spans="1:5" ht="14.25">
+      <c r="A21" s="3">
+        <v>8</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="19"/>
-      <c r="E21" s="20"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="19">
-        <v>9.0</v>
-      </c>
-      <c r="B22" s="20" t="s">
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" spans="1:5" ht="14.25">
+      <c r="A22" s="3">
+        <v>9</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D22" s="19"/>
-      <c r="E22" s="20"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="20">
-        <v>10.0</v>
-      </c>
-      <c r="B23" s="20" t="s">
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" spans="1:5" ht="14.25">
+      <c r="A23" s="3">
+        <v>10</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="19"/>
-      <c r="E23" s="20"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="19">
-        <v>11.0</v>
-      </c>
-      <c r="B24" s="20" t="s">
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" ht="14.25">
+      <c r="A24" s="3">
+        <v>11</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="19"/>
-      <c r="E24" s="20"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="20">
-        <v>12.0</v>
-      </c>
-      <c r="B25" s="20" t="s">
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" spans="1:5" ht="14.25">
+      <c r="A25" s="3">
+        <v>12</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D25" s="19"/>
-      <c r="E25" s="20"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="19">
-        <v>13.0</v>
-      </c>
-      <c r="B26" s="20" t="s">
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" spans="1:5" ht="14.25">
+      <c r="A26" s="3">
+        <v>13</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D26" s="19"/>
-      <c r="E26" s="20"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="20">
-        <v>14.0</v>
-      </c>
-      <c r="B27" s="20" t="s">
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" spans="1:5" ht="14.25">
+      <c r="A27" s="3">
+        <v>14</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="19"/>
-      <c r="E27" s="20"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="20">
-        <v>15.0</v>
-      </c>
-      <c r="B28" s="20" t="s">
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" spans="1:5" ht="14.25">
+      <c r="A28" s="3">
+        <v>15</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="19">
-        <v>16.0</v>
-      </c>
-      <c r="B29" s="20" t="s">
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" spans="1:5" ht="14.25">
+      <c r="A29" s="3">
+        <v>16</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="20">
-        <v>17.0</v>
-      </c>
-      <c r="B30" s="20" t="s">
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" spans="1:5" ht="14.25">
+      <c r="A30" s="3">
+        <v>17</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="20">
-        <v>18.0</v>
-      </c>
-      <c r="B31" s="20" t="s">
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" spans="1:5" ht="14.25">
+      <c r="A31" s="3">
+        <v>18</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D31" s="19"/>
-      <c r="E31" s="20" t="s">
+      <c r="D31" s="3"/>
+      <c r="E31" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="19">
-        <v>19.0</v>
-      </c>
-      <c r="B32" s="20" t="s">
+    <row r="32" spans="1:5" ht="14.25">
+      <c r="A32" s="3">
+        <v>19</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="20">
-        <v>20.0</v>
-      </c>
-      <c r="B33" s="20" t="s">
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+    </row>
+    <row r="33" spans="1:5" ht="14.25">
+      <c r="A33" s="3">
+        <v>20</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="20">
-        <v>21.0</v>
-      </c>
-      <c r="B34" s="20" t="s">
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+    </row>
+    <row r="34" spans="1:5" ht="14.25">
+      <c r="A34" s="3">
+        <v>21</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="19">
-        <v>22.0</v>
-      </c>
-      <c r="B35" s="20" t="s">
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+    </row>
+    <row r="35" spans="1:5" ht="14.25">
+      <c r="A35" s="3">
+        <v>22</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="16" t="s">
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+    </row>
+    <row r="36" spans="1:5" ht="14.25">
+      <c r="A36" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="18"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="20">
-        <v>1.0</v>
-      </c>
-      <c r="B37" s="20" t="s">
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="20"/>
+    </row>
+    <row r="37" spans="1:5" ht="14.25">
+      <c r="A37" s="3">
+        <v>1</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="20">
-        <v>2.0</v>
-      </c>
-      <c r="B38" s="20" t="s">
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+    </row>
+    <row r="38" spans="1:5" ht="14.25">
+      <c r="A38" s="3">
+        <v>2</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="20">
-        <v>3.0</v>
-      </c>
-      <c r="B39" s="20" t="s">
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+    </row>
+    <row r="39" spans="1:5" ht="14.25">
+      <c r="A39" s="3">
+        <v>3</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="20">
-        <v>4.0</v>
-      </c>
-      <c r="B40" s="20" t="s">
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+    </row>
+    <row r="40" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A40" s="3">
+        <v>4</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="20">
-        <v>5.0</v>
-      </c>
-      <c r="B41" s="20" t="s">
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A41" s="3">
+        <v>5</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="20">
-        <v>6.0</v>
-      </c>
-      <c r="B42" s="20" t="s">
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+    </row>
+    <row r="42" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A42" s="3">
+        <v>6</v>
+      </c>
+      <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="20">
-        <v>7.0</v>
-      </c>
-      <c r="B43" s="20" t="s">
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+    </row>
+    <row r="43" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A43" s="3">
+        <v>7</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="20">
-        <v>8.0</v>
-      </c>
-      <c r="B44" s="20" t="s">
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+    </row>
+    <row r="44" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A44" s="3">
+        <v>8</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="20">
-        <v>9.0</v>
-      </c>
-      <c r="B45" s="20" t="s">
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+    </row>
+    <row r="45" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A45" s="3">
+        <v>9</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="C45" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="20">
-        <v>10.0</v>
-      </c>
-      <c r="B46" s="20" t="s">
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A46" s="3">
+        <v>10</v>
+      </c>
+      <c r="B46" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C46" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="20">
-        <v>11.0</v>
-      </c>
-      <c r="B47" s="20" t="s">
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+    </row>
+    <row r="47" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A47" s="3">
+        <v>11</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C47" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="20">
-        <v>12.0</v>
-      </c>
-      <c r="B48" s="20" t="s">
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+    </row>
+    <row r="48" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A48" s="3">
+        <v>12</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C48" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D48" s="19"/>
-      <c r="E48" s="19"/>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="20">
-        <v>13.0</v>
-      </c>
-      <c r="B49" s="20" t="s">
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A49" s="3">
+        <v>13</v>
+      </c>
+      <c r="B49" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="C49" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="20">
-        <v>14.0</v>
-      </c>
-      <c r="B50" s="20" t="s">
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+    </row>
+    <row r="50" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A50" s="3">
+        <v>14</v>
+      </c>
+      <c r="B50" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D50" s="19"/>
-      <c r="E50" s="19"/>
-    </row>
-    <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="20">
-        <v>15.0</v>
-      </c>
-      <c r="B51" s="20" t="s">
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+    </row>
+    <row r="51" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A51" s="3">
+        <v>15</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D51" s="19"/>
-      <c r="E51" s="19"/>
-    </row>
-    <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="20">
-        <v>16.0</v>
-      </c>
-      <c r="B52" s="20" t="s">
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+    </row>
+    <row r="52" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A52" s="3">
+        <v>16</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="C52" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D52" s="19"/>
-      <c r="E52" s="19"/>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="20">
-        <v>17.0</v>
-      </c>
-      <c r="B53" s="20" t="s">
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+    </row>
+    <row r="53" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A53" s="3">
+        <v>17</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="C53" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D53" s="19"/>
-      <c r="E53" s="19"/>
-    </row>
-    <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="20">
-        <v>18.0</v>
-      </c>
-      <c r="B54" s="20" t="s">
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+    </row>
+    <row r="54" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A54" s="3">
+        <v>18</v>
+      </c>
+      <c r="B54" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C54" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D54" s="19"/>
-      <c r="E54" s="19"/>
-    </row>
-    <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="20">
-        <v>19.0</v>
-      </c>
-      <c r="B55" s="20" t="s">
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+    </row>
+    <row r="55" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A55" s="3">
+        <v>19</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C55" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D55" s="19"/>
-      <c r="E55" s="19"/>
-    </row>
-    <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="20">
-        <v>20.0</v>
-      </c>
-      <c r="B56" s="20" t="s">
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+    </row>
+    <row r="56" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A56" s="3">
+        <v>20</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C56" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D56" s="19"/>
-      <c r="E56" s="19"/>
-    </row>
-    <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="20">
-        <v>21.0</v>
-      </c>
-      <c r="B57" s="20" t="s">
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+    </row>
+    <row r="57" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A57" s="3">
+        <v>21</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C57" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-    </row>
-    <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="20">
-        <v>22.0</v>
-      </c>
-      <c r="B58" s="20" t="s">
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+    </row>
+    <row r="58" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A58" s="3">
+        <v>22</v>
+      </c>
+      <c r="B58" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="C58" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-    </row>
-    <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="20">
-        <v>23.0</v>
-      </c>
-      <c r="B59" s="20" t="s">
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+    </row>
+    <row r="59" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A59" s="3">
+        <v>23</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="C59" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-    </row>
-    <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="20">
-        <v>24.0</v>
-      </c>
-      <c r="B60" s="20" t="s">
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+    </row>
+    <row r="60" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A60" s="3">
+        <v>24</v>
+      </c>
+      <c r="B60" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-    </row>
-    <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="20">
-        <v>25.0</v>
-      </c>
-      <c r="B61" s="20" t="s">
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+    </row>
+    <row r="61" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A61" s="3">
+        <v>25</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D61" s="19"/>
-      <c r="E61" s="19"/>
-    </row>
-    <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="20">
-        <v>26.0</v>
-      </c>
-      <c r="B62" s="20" t="s">
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+    </row>
+    <row r="62" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A62" s="3">
+        <v>26</v>
+      </c>
+      <c r="B62" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C62" s="21" t="s">
+      <c r="C62" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D62" s="19"/>
-      <c r="E62" s="19"/>
-    </row>
-    <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="20">
-        <v>27.0</v>
-      </c>
-      <c r="B63" s="20" t="s">
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+    </row>
+    <row r="63" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A63" s="3">
+        <v>27</v>
+      </c>
+      <c r="B63" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="C63" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D63" s="19"/>
-      <c r="E63" s="19"/>
-    </row>
-    <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="20">
-        <v>28.0</v>
-      </c>
-      <c r="B64" s="20" t="s">
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+    </row>
+    <row r="64" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A64" s="3">
+        <v>28</v>
+      </c>
+      <c r="B64" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C64" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D64" s="19"/>
-      <c r="E64" s="19"/>
-    </row>
-    <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="20">
-        <v>29.0</v>
-      </c>
-      <c r="B65" s="20" t="s">
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+    </row>
+    <row r="65" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A65" s="3">
+        <v>29</v>
+      </c>
+      <c r="B65" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C65" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D65" s="19"/>
-      <c r="E65" s="19"/>
-    </row>
-    <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="20">
-        <v>30.0</v>
-      </c>
-      <c r="B66" s="20" t="s">
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+    </row>
+    <row r="66" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A66" s="3">
+        <v>30</v>
+      </c>
+      <c r="B66" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C66" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D66" s="19"/>
-      <c r="E66" s="19"/>
-    </row>
-    <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="20">
-        <v>31.0</v>
-      </c>
-      <c r="B67" s="20" t="s">
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+    </row>
+    <row r="67" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A67" s="3">
+        <v>31</v>
+      </c>
+      <c r="B67" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D67" s="19"/>
-      <c r="E67" s="20" t="s">
+      <c r="D67" s="3"/>
+      <c r="E67" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="20">
-        <v>32.0</v>
-      </c>
-      <c r="B68" s="20" t="s">
+    <row r="68" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A68" s="3">
+        <v>32</v>
+      </c>
+      <c r="B68" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="C68" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D68" s="19"/>
-      <c r="E68" s="20" t="s">
+      <c r="D68" s="3"/>
+      <c r="E68" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="20">
-        <v>33.0</v>
-      </c>
-      <c r="B69" s="20" t="s">
+    <row r="69" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A69" s="3">
+        <v>33</v>
+      </c>
+      <c r="B69" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="C69" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D69" s="19"/>
-      <c r="E69" s="20" t="s">
+      <c r="D69" s="3"/>
+      <c r="E69" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="20">
-        <v>34.0</v>
-      </c>
-      <c r="B70" s="20" t="s">
+    <row r="70" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A70" s="3">
+        <v>34</v>
+      </c>
+      <c r="B70" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D70" s="19"/>
-      <c r="E70" s="20" t="s">
+      <c r="D70" s="3"/>
+      <c r="E70" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="20">
-        <v>35.0</v>
-      </c>
-      <c r="B71" s="20" t="s">
+    <row r="71" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A71" s="3">
+        <v>35</v>
+      </c>
+      <c r="B71" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="C71" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D71" s="19"/>
-      <c r="E71" s="20" t="s">
+      <c r="D71" s="3"/>
+      <c r="E71" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="20">
-        <v>36.0</v>
-      </c>
-      <c r="B72" s="20" t="s">
+    <row r="72" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A72" s="3">
+        <v>36</v>
+      </c>
+      <c r="B72" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C72" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D72" s="19"/>
-      <c r="E72" s="20" t="s">
+      <c r="D72" s="3"/>
+      <c r="E72" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="20">
-        <v>37.0</v>
-      </c>
-      <c r="B73" s="20" t="s">
+    <row r="73" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A73" s="3">
+        <v>37</v>
+      </c>
+      <c r="B73" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="C73" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D73" s="19"/>
-      <c r="E73" s="20" t="s">
+      <c r="D73" s="3"/>
+      <c r="E73" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="20">
-        <v>38.0</v>
-      </c>
-      <c r="B74" s="20" t="s">
+    <row r="74" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A74" s="3">
+        <v>38</v>
+      </c>
+      <c r="B74" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C74" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D74" s="19"/>
-      <c r="E74" s="20" t="s">
+      <c r="D74" s="3"/>
+      <c r="E74" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="20">
-        <v>39.0</v>
-      </c>
-      <c r="B75" s="20" t="s">
+    <row r="75" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A75" s="3">
+        <v>39</v>
+      </c>
+      <c r="B75" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C75" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D75" s="19"/>
-      <c r="E75" s="20" t="s">
+      <c r="D75" s="3"/>
+      <c r="E75" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="20">
-        <v>40.0</v>
-      </c>
-      <c r="B76" s="20" t="s">
+    <row r="76" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A76" s="3">
+        <v>40</v>
+      </c>
+      <c r="B76" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="C76" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D76" s="19"/>
-      <c r="E76" s="20" t="s">
+      <c r="D76" s="3"/>
+      <c r="E76" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="22" t="s">
+    <row r="77" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A77" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="B77" s="17"/>
-      <c r="C77" s="17"/>
-      <c r="D77" s="17"/>
-      <c r="E77" s="18"/>
-    </row>
-    <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="20">
-        <v>1.0</v>
-      </c>
-      <c r="B78" s="20" t="s">
+      <c r="B77" s="19"/>
+      <c r="C77" s="19"/>
+      <c r="D77" s="19"/>
+      <c r="E77" s="20"/>
+    </row>
+    <row r="78" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A78" s="3">
+        <v>1</v>
+      </c>
+      <c r="B78" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C78" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D78" s="19"/>
-      <c r="E78" s="19"/>
-    </row>
-    <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="20">
-        <v>2.0</v>
-      </c>
-      <c r="B79" s="20" t="s">
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+    </row>
+    <row r="79" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A79" s="3">
+        <v>2</v>
+      </c>
+      <c r="B79" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="C79" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D79" s="19"/>
-      <c r="E79" s="19"/>
-    </row>
-    <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="20">
-        <v>3.0</v>
-      </c>
-      <c r="B80" s="20" t="s">
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+    </row>
+    <row r="80" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A80" s="3">
+        <v>3</v>
+      </c>
+      <c r="B80" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="C80" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D80" s="19"/>
-      <c r="E80" s="19"/>
-    </row>
-    <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="20">
-        <v>4.0</v>
-      </c>
-      <c r="B81" s="20" t="s">
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+    </row>
+    <row r="81" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A81" s="3">
+        <v>4</v>
+      </c>
+      <c r="B81" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="C81" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D81" s="19"/>
-      <c r="E81" s="19"/>
-    </row>
-    <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="20">
-        <v>5.0</v>
-      </c>
-      <c r="B82" s="20" t="s">
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+    </row>
+    <row r="82" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A82" s="3">
+        <v>5</v>
+      </c>
+      <c r="B82" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="C82" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D82" s="19"/>
-      <c r="E82" s="19"/>
-    </row>
-    <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="20">
-        <v>6.0</v>
-      </c>
-      <c r="B83" s="20" t="s">
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+    </row>
+    <row r="83" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A83" s="3">
+        <v>6</v>
+      </c>
+      <c r="B83" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C83" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D83" s="19"/>
-      <c r="E83" s="19"/>
-    </row>
-    <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="20">
-        <v>7.0</v>
-      </c>
-      <c r="B84" s="20" t="s">
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+    </row>
+    <row r="84" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A84" s="3">
+        <v>7</v>
+      </c>
+      <c r="B84" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C84" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D84" s="19"/>
-      <c r="E84" s="19"/>
-    </row>
-    <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="20">
-        <v>8.0</v>
-      </c>
-      <c r="B85" s="20" t="s">
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+    </row>
+    <row r="85" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A85" s="3">
+        <v>8</v>
+      </c>
+      <c r="B85" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C85" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D85" s="19"/>
-      <c r="E85" s="19"/>
-    </row>
-    <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="20">
-        <v>9.0</v>
-      </c>
-      <c r="B86" s="20" t="s">
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+    </row>
+    <row r="86" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A86" s="3">
+        <v>9</v>
+      </c>
+      <c r="B86" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C86" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D86" s="19"/>
-      <c r="E86" s="20" t="s">
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+    </row>
+    <row r="87" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A87" s="3">
+        <v>10</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="20">
-        <v>10.0</v>
-      </c>
-      <c r="B87" s="20" t="s">
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+    </row>
+    <row r="88" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A88" s="3">
+        <v>11</v>
+      </c>
+      <c r="B88" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C88" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D87" s="19"/>
-      <c r="E87" s="19"/>
-    </row>
-    <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="20">
-        <v>11.0</v>
-      </c>
-      <c r="B88" s="20" t="s">
+      <c r="D88" s="3"/>
+    </row>
+    <row r="89" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A89" s="3">
+        <v>12</v>
+      </c>
+      <c r="B89" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C88" s="2" t="s">
+      <c r="C89" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D88" s="19"/>
-      <c r="E88" s="19"/>
-    </row>
-    <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="20">
-        <v>12.0</v>
-      </c>
-      <c r="B89" s="20" t="s">
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+    </row>
+    <row r="90" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A90" s="3">
+        <v>13</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A91" s="3">
+        <v>14</v>
+      </c>
+      <c r="B91" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C89" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="D89" s="19"/>
-      <c r="E89" s="19"/>
-    </row>
-    <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="20">
-        <v>13.0</v>
-      </c>
-      <c r="B90" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D90" s="19"/>
-      <c r="E90" s="20" t="s">
+      <c r="C91" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+    </row>
+    <row r="92" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A92" s="3">
+        <v>15</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="20">
-        <v>14.0</v>
-      </c>
-      <c r="B91" s="20" t="s">
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+    </row>
+    <row r="93" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A93" s="3">
+        <v>16</v>
+      </c>
+      <c r="B93" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C91" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D91" s="19"/>
-      <c r="E91" s="19"/>
-    </row>
-    <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="20">
-        <v>15.0</v>
-      </c>
-      <c r="B92" s="20" t="s">
+      <c r="C93" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+    </row>
+    <row r="94" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A94" s="3">
+        <v>17</v>
+      </c>
+      <c r="B94" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C92" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="D92" s="19"/>
-      <c r="E92" s="19"/>
-    </row>
-    <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="20">
-        <v>16.0</v>
-      </c>
-      <c r="B93" s="20" t="s">
+      <c r="C94" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+    </row>
+    <row r="95" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A95" s="3">
+        <v>18</v>
+      </c>
+      <c r="B95" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C93" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D93" s="19"/>
-      <c r="E93" s="19"/>
-    </row>
-    <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="20">
-        <v>17.0</v>
-      </c>
-      <c r="B94" s="20" t="s">
+      <c r="C95" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+    </row>
+    <row r="96" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A96" s="3">
+        <v>19</v>
+      </c>
+      <c r="B96" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C94" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D94" s="19"/>
-      <c r="E94" s="19"/>
-    </row>
-    <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="20">
-        <v>18.0</v>
-      </c>
-      <c r="B95" s="20" t="s">
+      <c r="C96" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+    </row>
+    <row r="97" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A97" s="3">
+        <v>20</v>
+      </c>
+      <c r="B97" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C95" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D95" s="19"/>
-      <c r="E95" s="19"/>
-    </row>
-    <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="20">
-        <v>19.0</v>
-      </c>
-      <c r="B96" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="C96" s="2" t="s">
+      <c r="C97" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D96" s="19"/>
-      <c r="E96" s="19"/>
-    </row>
-    <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="20">
-        <v>20.0</v>
-      </c>
-      <c r="B97" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="C97" s="2" t="s">
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+    </row>
+    <row r="98" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A98" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="D97" s="19"/>
-      <c r="E97" s="19"/>
-    </row>
-    <row r="98" ht="15.75" customHeight="1">
-      <c r="A98" s="16" t="s">
+      <c r="B98" s="19"/>
+      <c r="C98" s="19"/>
+      <c r="D98" s="19"/>
+      <c r="E98" s="20"/>
+    </row>
+    <row r="99" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A99" s="3"/>
+      <c r="B99" s="3"/>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B98" s="17"/>
-      <c r="C98" s="17"/>
-      <c r="D98" s="17"/>
-      <c r="E98" s="18"/>
-    </row>
-    <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="19"/>
-      <c r="B99" s="19"/>
-      <c r="C99" s="19"/>
-      <c r="D99" s="19"/>
-      <c r="E99" s="19" t="s">
+    </row>
+    <row r="100" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A100" s="3">
+        <v>1</v>
+      </c>
+      <c r="B100" s="5" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="100" ht="15.75" customHeight="1">
-      <c r="A100" s="20">
-        <v>1.0</v>
-      </c>
-      <c r="B100" s="23" t="s">
+      <c r="C100" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C100" s="19" t="s">
+      <c r="D100" s="3"/>
+      <c r="E100" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="D100" s="19"/>
-      <c r="E100" s="20" t="s">
+    </row>
+    <row r="101" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A101" s="3">
+        <v>2</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C101" s="3" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="20">
-        <v>2.0</v>
-      </c>
-      <c r="B101" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="C101" s="20" t="s">
+      <c r="D101" s="3"/>
+      <c r="E101" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D101" s="19"/>
-      <c r="E101" s="20" t="s">
+    </row>
+    <row r="102" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A102" s="3">
+        <v>3</v>
+      </c>
+      <c r="B102" s="5" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="102" ht="15.75" customHeight="1">
-      <c r="A102" s="20">
-        <v>3.0</v>
-      </c>
-      <c r="B102" s="23" t="s">
+      <c r="C102" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C102" s="19" t="s">
+      <c r="D102" s="3"/>
+      <c r="E102" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D102" s="19"/>
-      <c r="E102" s="20" t="s">
+    </row>
+    <row r="103" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A103" s="3">
+        <v>4</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C103" s="3" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="20">
-        <v>4.0</v>
-      </c>
-      <c r="B103" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="C103" s="20" t="s">
+      <c r="D103" s="3"/>
+      <c r="E103" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="D103" s="19"/>
-      <c r="E103" s="20" t="s">
+    </row>
+    <row r="104" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A104" s="3">
+        <v>5</v>
+      </c>
+      <c r="B104" s="5" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="104" ht="15.75" customHeight="1">
-      <c r="A104" s="20">
-        <v>5.0</v>
-      </c>
-      <c r="B104" s="23" t="s">
+      <c r="C104" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="C104" s="20" t="s">
+      <c r="D104" s="3"/>
+      <c r="E104" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="D104" s="19"/>
-      <c r="E104" s="20" t="s">
+    </row>
+    <row r="105" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A105" s="3">
+        <v>6</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C105" s="3" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="20">
-        <v>6.0</v>
-      </c>
-      <c r="B105" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="C105" s="19" t="s">
+      <c r="D105" s="3"/>
+      <c r="E105" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D105" s="19"/>
-      <c r="E105" s="20" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
+    </row>
+    <row r="106" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="107" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="108" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="109" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="110" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="111" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="112" spans="1:5" ht="15.75" customHeight="1"/>
     <row r="113" ht="15.75" customHeight="1"/>
     <row r="114" ht="15.75" customHeight="1"/>
     <row r="115" ht="15.75" customHeight="1"/>
@@ -3303,32 +3392,30 @@
     <row r="1071" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A98:E98"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E10"/>
     <mergeCell ref="F5:I10"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A77:E77"/>
-    <mergeCell ref="A98:E98"/>
   </mergeCells>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B78:B97">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B78:B97" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Bukan Kerentanan,Kerentanan,-"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B14:B35">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B14:B35" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Aset,Bukan Aset,-"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B100:B105">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B100:B105" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Kontrol (Akses),Kontrol (Awareness),Kontrol (Logging),-"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B37:B76">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B37:B76" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Ancaman,Bukan Ancaman,-"</formula1>
     </dataValidation>
   </dataValidations>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>